<commit_message>
Update AMS weekly data and processed ads reports
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/White_Mulberry/business_report_week18.xlsx
+++ b/data/ams_weekly_data/White_Mulberry/business_report_week18.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Week 17\Week 18\ams_weekly_data\White_Mulberry\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Laptop\D\Nitesh\Weekly Report - B2B + B2C\FastAPI\data\ams_weekly_data\White_Mulberry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A865158-CD76-4EA3-90DC-73641D6A60F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802E0594-CB94-4870-AEBB-8B3D0C788899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2989,11 +2989,11 @@
       <c r="E29" t="s">
         <v>118</v>
       </c>
-      <c r="P29" s="6">
+      <c r="P29">
+        <v>68</v>
+      </c>
+      <c r="T29" s="6">
         <v>167061.04</v>
-      </c>
-      <c r="T29">
-        <v>68</v>
       </c>
     </row>
     <row r="30" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3012,11 +3012,11 @@
       <c r="E30" t="s">
         <v>110</v>
       </c>
-      <c r="P30" s="6">
+      <c r="P30">
+        <v>11</v>
+      </c>
+      <c r="T30" s="6">
         <v>25626.26</v>
-      </c>
-      <c r="T30">
-        <v>11</v>
       </c>
     </row>
     <row r="31" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3035,11 +3035,11 @@
       <c r="E31" t="s">
         <v>122</v>
       </c>
-      <c r="P31" s="6">
+      <c r="P31">
+        <v>8</v>
+      </c>
+      <c r="T31" s="6">
         <v>21010.17</v>
-      </c>
-      <c r="T31">
-        <v>8</v>
       </c>
     </row>
     <row r="32" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3058,11 +3058,11 @@
       <c r="E32" t="s">
         <v>102</v>
       </c>
-      <c r="P32" s="6">
+      <c r="P32">
+        <v>10</v>
+      </c>
+      <c r="T32" s="6">
         <v>16940.64</v>
-      </c>
-      <c r="T32">
-        <v>10</v>
       </c>
     </row>
     <row r="33" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3081,11 +3081,11 @@
       <c r="E33" t="s">
         <v>114</v>
       </c>
-      <c r="P33" s="6">
+      <c r="P33">
+        <v>3</v>
+      </c>
+      <c r="T33" s="6">
         <v>11946.6</v>
-      </c>
-      <c r="T33">
-        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3104,11 +3104,11 @@
       <c r="E34" t="s">
         <v>130</v>
       </c>
-      <c r="P34" s="6">
+      <c r="P34">
+        <v>6</v>
+      </c>
+      <c r="T34" s="6">
         <v>10164.41</v>
-      </c>
-      <c r="T34">
-        <v>6</v>
       </c>
     </row>
     <row r="35" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -3127,11 +3127,11 @@
       <c r="E35" t="s">
         <v>26</v>
       </c>
-      <c r="P35" s="6">
+      <c r="P35">
+        <v>-1</v>
+      </c>
+      <c r="T35" s="6">
         <v>-1355.08</v>
-      </c>
-      <c r="T35">
-        <v>-1</v>
       </c>
     </row>
     <row r="36" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>